<commit_message>
Hide calc on check page
</commit_message>
<xml_diff>
--- a/bill-checker-demo.xlsx
+++ b/bill-checker-demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alinaaleks\Downloads\GitHub\bill-checker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553D1359-A41E-40EE-887F-D6392D611513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0F4EBE-4F58-44EE-B5E3-4E7EE5455264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -521,16 +521,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="yyyy\-mm"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000"/>
-    <numFmt numFmtId="170" formatCode="#,##0.0000"/>
-    <numFmt numFmtId="172" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="#,##0.000"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -578,6 +579,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -904,9 +912,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1116,9 +1125,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1131,13 +1137,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1155,17 +1155,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1176,13 +1167,10 @@
     <xf numFmtId="1" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1191,62 +1179,14 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="9" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1269,90 +1209,82 @@
     <xf numFmtId="4" fontId="0" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="3" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="3" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="9" borderId="17" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="9" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="8" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="105">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="62">
     <dxf>
       <font>
         <color theme="9" tint="-0.499984740745262"/>
@@ -1391,319 +1323,9 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1805,6 +1427,39 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
       <alignment vertical="center"/>
     </dxf>
     <dxf>
@@ -1863,39 +1518,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
@@ -4968,8 +4590,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5826397" y="123009"/>
-              <a:ext cx="4503963" cy="2947488"/>
+              <a:off x="5841637" y="124279"/>
+              <a:ext cx="4505233" cy="2928438"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -5335,6 +4957,193 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4747A43B-033B-44E1-A183-5A9895611AE7}" name="отклонения по месяцам" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" outline="1" outlineData="1" compactData="0" multipleFieldFilters="0">
+  <location ref="A2:F5" firstHeaderRow="0" firstDataRow="1" firstDataCol="2"/>
+  <pivotFields count="22">
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" numFmtId="14" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" showAll="0">
+      <items count="4">
+        <item m="1" x="2"/>
+        <item m="1" x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" showAll="0">
+      <items count="14">
+        <item m="1" x="4"/>
+        <item m="1" x="3"/>
+        <item m="1" x="2"/>
+        <item m="1" x="1"/>
+        <item m="1" x="12"/>
+        <item m="1" x="11"/>
+        <item m="1" x="10"/>
+        <item m="1" x="9"/>
+        <item m="1" x="8"/>
+        <item m="1" x="7"/>
+        <item m="1" x="6"/>
+        <item m="1" x="5"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" compact="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField dataField="1" compact="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="17"/>
+    <field x="19"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+  </colItems>
+  <dataFields count="4">
+    <dataField name="План (начисления)" fld="10" baseField="17" baseItem="0"/>
+    <dataField name="Факт (начисления)" fld="4" baseField="17" baseItem="0" numFmtId="4"/>
+    <dataField name="Отклонение (руб)" fld="20" baseField="17" baseItem="0"/>
+    <dataField name="Отклонение (%)" fld="21" baseField="17" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <formats count="11">
+    <format dxfId="37">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="36">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="35">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="34">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="33">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea field="19" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
+    </format>
+    <format dxfId="31">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="4">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="30">
+      <pivotArea field="19" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
+    </format>
+    <format dxfId="29">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="4">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="28">
+      <pivotArea field="19" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
+    </format>
+    <format dxfId="27">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="4">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleMedium9" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{78231426-3946-4FAE-A363-072197D8DAF2}" name="PivotTable36" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" rowHeaderCaption="Месяц">
   <location ref="AA4:AB6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
@@ -5428,7 +5237,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{83BBBD9A-9D48-47B7-8427-426296D86302}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B27:F31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
@@ -5532,10 +5341,10 @@
     <dataField name="Отклонение (%)" fld="21" baseField="13" baseItem="1" numFmtId="10"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="75">
+    <format dxfId="43">
       <pivotArea field="17" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="42">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -5547,10 +5356,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="41">
       <pivotArea field="17" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="72">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -5562,10 +5371,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="71">
+    <format dxfId="39">
       <pivotArea field="17" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="70">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="4">
@@ -5590,7 +5399,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{36734D62-F45A-43F2-8842-27AFF588CCB5}" name="отклонения по услугам" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" updatedVersion="8" minRefreshableVersion="3" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" rowHeaderCaption="Услуга">
   <location ref="U2:W6" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="22">
@@ -5663,7 +5472,7 @@
     <dataField name="Факт (начисления)" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="18">
-    <format dxfId="93">
+    <format dxfId="61">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5675,10 +5484,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="92">
+    <format dxfId="60">
       <pivotArea field="17" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="91">
+    <format dxfId="59">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="17" count="1">
@@ -5687,7 +5496,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1">
@@ -5699,7 +5508,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="57">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5711,13 +5520,13 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="56">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="87">
+    <format dxfId="55">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="54">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2" selected="0">
@@ -5730,7 +5539,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5742,31 +5551,31 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="52">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="83">
+    <format dxfId="51">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="82">
+    <format dxfId="50">
       <pivotArea field="17" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="81">
+    <format dxfId="49">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="80">
+    <format dxfId="48">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="79">
+    <format dxfId="47">
       <pivotArea field="-2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="1"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="46">
       <pivotArea field="17" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="77">
+    <format dxfId="45">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="17" count="1">
@@ -5862,227 +5671,40 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4747A43B-033B-44E1-A183-5A9895611AE7}" name="отклонения по месяцам" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" outline="1" outlineData="1" compactData="0" multipleFieldFilters="0">
-  <location ref="A2:F5" firstHeaderRow="0" firstDataRow="1" firstDataCol="2"/>
-  <pivotFields count="22">
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" numFmtId="14" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" showAll="0">
-      <items count="4">
-        <item m="1" x="2"/>
-        <item m="1" x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" showAll="0">
-      <items count="14">
-        <item m="1" x="4"/>
-        <item m="1" x="3"/>
-        <item m="1" x="2"/>
-        <item m="1" x="1"/>
-        <item m="1" x="12"/>
-        <item m="1" x="11"/>
-        <item m="1" x="10"/>
-        <item m="1" x="9"/>
-        <item m="1" x="8"/>
-        <item m="1" x="7"/>
-        <item m="1" x="6"/>
-        <item m="1" x="5"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" compact="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" compact="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="17"/>
-    <field x="19"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-  </colItems>
-  <dataFields count="4">
-    <dataField name="План (начисления)" fld="10" baseField="17" baseItem="0"/>
-    <dataField name="Факт (начисления)" fld="4" baseField="17" baseItem="0" numFmtId="4"/>
-    <dataField name="Отклонение (руб)" fld="20" baseField="17" baseItem="0"/>
-    <dataField name="Отклонение (%)" fld="21" baseField="17" baseItem="0" numFmtId="10"/>
-  </dataFields>
-  <formats count="11">
-    <format dxfId="104">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="103">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="102">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="101">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="100">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="99">
-      <pivotArea field="19" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
-    </format>
-    <format dxfId="98">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="97">
-      <pivotArea field="19" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
-    </format>
-    <format dxfId="96">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="95">
-      <pivotArea field="19" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="1"/>
-    </format>
-    <format dxfId="94">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="4">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleMedium9" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{038A7D06-120E-408B-AEDA-813F2FAAD501}" name="Table2" displayName="Table2" ref="A1:T2" insertRow="1" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{038A7D06-120E-408B-AEDA-813F2FAAD501}" name="Table2" displayName="Table2" ref="A1:T2" insertRow="1" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:T2" xr:uid="{038A7D06-120E-408B-AEDA-813F2FAAD501}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{A040E5F1-B940-434F-8642-3D7965B0C906}" name="услуга" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{F1E9BBF3-FF65-4BCE-A746-A764AA053336}" name="ед_изм" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{95BCA9F7-93A8-474A-B486-B60193571EE3}" name="объем_квит" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{68D5AF23-9C08-4C25-A70E-D5B9C5258B85}" name="тариф_квит" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{1AE3F8D2-8628-41AA-B125-5D9318037FFC}" name="начислено_квит" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{2352EB12-E5C2-4AD6-8516-1C5A276F0128}" name="объем_откл" dataDxfId="62"/>
-    <tableColumn id="7" xr3:uid="{7BC866F5-0902-4D0A-9F28-F44EC965920C}" name="тариф_откл" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{DCE0FDDD-E687-4FB1-A515-511A0D4227D7}" name="начислено_откл" dataDxfId="60"/>
-    <tableColumn id="9" xr3:uid="{ABA713D2-6A48-414E-8866-3C6F39D5A490}" name="объем_расчет" dataDxfId="59"/>
-    <tableColumn id="10" xr3:uid="{EB157C1F-294F-4DFA-B0C3-E5402FF488C6}" name="тариф_расчет" dataDxfId="58"/>
-    <tableColumn id="11" xr3:uid="{16FD8211-F0B8-47DC-B4C9-EE5186864112}" name="насчислено_расчет" dataDxfId="57"/>
-    <tableColumn id="12" xr3:uid="{E9403770-B09D-40E2-BEFE-72B760354FEB}" name="норматив" dataDxfId="56"/>
-    <tableColumn id="13" xr3:uid="{5E21BED0-908D-4682-8E01-9D5911F61AB9}" name="период" dataDxfId="55"/>
-    <tableColumn id="14" xr3:uid="{6C555CCE-FDE0-4600-A16A-E7977D4C1331}" name="поставщик" dataDxfId="54"/>
-    <tableColumn id="18" xr3:uid="{70B0664C-2BB9-44F5-A956-B8CFF607EBD0}" name="начислено_откл%" dataDxfId="53">
+    <tableColumn id="1" xr3:uid="{A040E5F1-B940-434F-8642-3D7965B0C906}" name="услуга" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{F1E9BBF3-FF65-4BCE-A746-A764AA053336}" name="ед_изм" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{95BCA9F7-93A8-474A-B486-B60193571EE3}" name="объем_квит" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{68D5AF23-9C08-4C25-A70E-D5B9C5258B85}" name="тариф_квит" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{1AE3F8D2-8628-41AA-B125-5D9318037FFC}" name="начислено_квит" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{2352EB12-E5C2-4AD6-8516-1C5A276F0128}" name="объем_откл" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{7BC866F5-0902-4D0A-9F28-F44EC965920C}" name="тариф_откл" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{DCE0FDDD-E687-4FB1-A515-511A0D4227D7}" name="начислено_откл" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{ABA713D2-6A48-414E-8866-3C6F39D5A490}" name="объем_расчет" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{EB157C1F-294F-4DFA-B0C3-E5402FF488C6}" name="тариф_расчет" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{16FD8211-F0B8-47DC-B4C9-EE5186864112}" name="насчислено_расчет" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{E9403770-B09D-40E2-BEFE-72B760354FEB}" name="норматив" dataDxfId="13"/>
+    <tableColumn id="13" xr3:uid="{5E21BED0-908D-4682-8E01-9D5911F61AB9}" name="период" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{6C555CCE-FDE0-4600-A16A-E7977D4C1331}" name="поставщик" dataDxfId="11"/>
+    <tableColumn id="18" xr3:uid="{70B0664C-2BB9-44F5-A956-B8CFF607EBD0}" name="начислено_откл%" dataDxfId="10">
       <calculatedColumnFormula>IF(Table2[[#This Row],[начислено_откл]]=0,0,(Table2[[#This Row],[начислено_квит]]-Table2[[#This Row],[насчислено_расчет]])/Table2[[#This Row],[насчислено_расчет]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{725C5E98-3B75-474D-9C6F-E06942598B1D}" name="положит_откл" dataDxfId="52">
+    <tableColumn id="19" xr3:uid="{725C5E98-3B75-474D-9C6F-E06942598B1D}" name="положит_откл" dataDxfId="9">
       <calculatedColumnFormula>IF(Table2[[#This Row],[начислено_откл]]&gt;0,Table2[[#This Row],[начислено_откл]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{307D926C-82F4-46F4-AC93-88CE44B6AD40}" name="отриц_откл" dataDxfId="51">
+    <tableColumn id="20" xr3:uid="{307D926C-82F4-46F4-AC93-88CE44B6AD40}" name="отриц_откл" dataDxfId="8">
       <calculatedColumnFormula>IF(Table2[[#This Row],[начислено_откл]]&lt;0,Table2[[#This Row],[начислено_откл]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{5780D1EA-A409-449C-BCA3-DC86372888EC}" name="год" dataDxfId="50">
+    <tableColumn id="15" xr3:uid="{5780D1EA-A409-449C-BCA3-DC86372888EC}" name="год" dataDxfId="7">
       <calculatedColumnFormula>YEAR(M2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{3889E082-3447-4F9E-A275-7FE45FCFD6FB}" name="месяц_№" dataDxfId="49">
+    <tableColumn id="16" xr3:uid="{3889E082-3447-4F9E-A275-7FE45FCFD6FB}" name="месяц_№" dataDxfId="6">
       <calculatedColumnFormula>MONTH(M2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{E6E9DC5E-485F-4A72-A2BF-41BAB4F90D1B}" name="месяц" dataDxfId="48">
+    <tableColumn id="17" xr3:uid="{E6E9DC5E-485F-4A72-A2BF-41BAB4F90D1B}" name="месяц" dataDxfId="5">
       <calculatedColumnFormula>CHOOSE(S2,"январь","февраль","март","апрель","май","июнь","июль","август","сентябрь","октябрь","ноябрь","декабрь")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6408,20 +6030,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8273ECE3-36C8-4C46-AC21-390A7CBD00EF}">
   <dimension ref="A1:N32"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.26953125" style="3" customWidth="1"/>
     <col min="2" max="2" width="11.36328125" style="3" customWidth="1"/>
     <col min="3" max="3" width="9" style="3" customWidth="1"/>
     <col min="4" max="4" width="11" style="3" customWidth="1"/>
     <col min="5" max="5" width="11.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="11.26953125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" style="3" customWidth="1"/>
-    <col min="9" max="10" width="11.26953125" style="3" customWidth="1"/>
+    <col min="6" max="7" width="11.26953125" style="3" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="11.36328125" style="3" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="11.26953125" style="3" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="11.26953125" style="3" customWidth="1"/>
     <col min="11" max="11" width="11.36328125" style="3" customWidth="1"/>
     <col min="12" max="12" width="14.90625" style="3" customWidth="1"/>
     <col min="13" max="13" width="11.26953125" style="3" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="16.7265625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="16.7265625" style="3" hidden="1" customWidth="1"/>
     <col min="15" max="15" width="59.1796875" style="3" customWidth="1"/>
     <col min="16" max="16384" width="9.1796875" style="3"/>
   </cols>
@@ -6453,7 +6076,7 @@
       <c r="A4" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="77">
+      <c r="B4" s="76">
         <f>info!B7</f>
         <v>55.2</v>
       </c>
@@ -6463,7 +6086,7 @@
       <c r="A5" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B5" s="75">
+      <c r="B5" s="74">
         <f>info!B6</f>
         <v>2</v>
       </c>
@@ -6474,21 +6097,21 @@
     <row r="7" spans="1:14" s="5" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
-      <c r="C7" s="87" t="s">
+      <c r="C7" s="101" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="88"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="99" t="s">
+      <c r="D7" s="102"/>
+      <c r="E7" s="103"/>
+      <c r="F7" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="G7" s="100"/>
-      <c r="H7" s="101"/>
-      <c r="I7" s="114" t="s">
+      <c r="G7" s="105"/>
+      <c r="H7" s="106"/>
+      <c r="I7" s="107" t="s">
         <v>155</v>
       </c>
-      <c r="J7" s="115"/>
-      <c r="K7" s="116"/>
+      <c r="J7" s="108"/>
+      <c r="K7" s="109"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
     </row>
@@ -6499,34 +6122,34 @@
       <c r="B8" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="90" t="s">
+      <c r="C8" s="84" t="s">
         <v>40</v>
       </c>
       <c r="D8" s="72" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="91" t="s">
+      <c r="E8" s="85" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="102" t="s">
+      <c r="F8" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="74" t="s">
+      <c r="G8" s="73" t="s">
         <v>41</v>
       </c>
-      <c r="H8" s="103" t="s">
+      <c r="H8" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="I8" s="117" t="s">
+      <c r="I8" s="94" t="s">
         <v>40</v>
       </c>
       <c r="J8" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="K8" s="118" t="s">
+      <c r="K8" s="95" t="s">
         <v>42</v>
       </c>
-      <c r="L8" s="113" t="s">
+      <c r="L8" s="93" t="s">
         <v>138</v>
       </c>
       <c r="M8" s="8" t="s">
@@ -6543,28 +6166,28 @@
       <c r="B9" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="92">
+      <c r="C9" s="86">
         <v>204</v>
       </c>
-      <c r="D9" s="83">
+      <c r="D9" s="80">
         <v>4.2</v>
       </c>
-      <c r="E9" s="93">
+      <c r="E9" s="112">
         <v>856.80000000000007</v>
       </c>
-      <c r="F9" s="104">
+      <c r="F9" s="116">
         <f>IFERROR(INDEX(usage!B:B, MATCH(CHECK!$B$3, usage!A:A, 0)) - INDEX(usage!B:B, MATCH(CHECK!$B$1, usage!A:A, 0)),"")</f>
         <v>201</v>
       </c>
-      <c r="G9" s="73">
+      <c r="G9" s="117">
         <f>IF(F9&lt;M9, INDEX(tariffs!2:2, MATCH(CHECK!$B$3,tariffs!$1:$1, 0)), INDEX(tariffs!3:3, MATCH(CHECK!$B$3,tariffs!$1:$1, 0)))</f>
         <v>4.2</v>
       </c>
-      <c r="H9" s="105">
+      <c r="H9" s="114">
         <f>IFERROR(F9*G9,"")</f>
         <v>844.2</v>
       </c>
-      <c r="I9" s="119">
+      <c r="I9" s="96">
         <f>IF(C9="", "", C9-F9)</f>
         <v>3</v>
       </c>
@@ -6572,7 +6195,7 @@
         <f t="shared" ref="J9:K24" si="0">IF(D9="", "", D9-G9)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="120">
+      <c r="K9" s="97">
         <f t="shared" si="0"/>
         <v>12.600000000000023</v>
       </c>
@@ -6596,28 +6219,28 @@
       <c r="B10" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="94">
+      <c r="C10" s="87">
         <v>4.597999999999999</v>
       </c>
-      <c r="D10" s="83">
+      <c r="D10" s="80">
         <v>62.98</v>
       </c>
-      <c r="E10" s="93">
+      <c r="E10" s="112">
         <v>289.58203999999995</v>
       </c>
-      <c r="F10" s="106">
+      <c r="F10" s="118">
         <f>IFERROR(INDEX(usage!C:C, MATCH(CHECK!$B$3, usage!A:A, 0)) - INDEX(usage!C:C, MATCH(CHECK!$B$1, usage!A:A, 0)),"")</f>
         <v>4.597999999999999</v>
       </c>
-      <c r="G10" s="73">
+      <c r="G10" s="117">
         <f>INDEX(tariffs!4:4, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>62.98</v>
       </c>
-      <c r="H10" s="105">
+      <c r="H10" s="114">
         <f t="shared" ref="H10:H24" si="1">IFERROR(F10*G10,"")</f>
         <v>289.58203999999995</v>
       </c>
-      <c r="I10" s="119">
+      <c r="I10" s="96">
         <f t="shared" ref="I10:I24" si="2">IF(C10="", "", C10-F10)</f>
         <v>0</v>
       </c>
@@ -6625,7 +6248,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K10" s="120">
+      <c r="K10" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6646,28 +6269,28 @@
       <c r="B11" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="94">
+      <c r="C11" s="87">
         <v>4.597999999999999</v>
       </c>
-      <c r="D11" s="83">
+      <c r="D11" s="80">
         <v>44.12</v>
       </c>
-      <c r="E11" s="93">
+      <c r="E11" s="112">
         <v>202.86375999999996</v>
       </c>
-      <c r="F11" s="106">
+      <c r="F11" s="118">
         <f>F10</f>
         <v>4.597999999999999</v>
       </c>
-      <c r="G11" s="73">
+      <c r="G11" s="117">
         <f>INDEX(tariffs!5:5, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>44.12</v>
       </c>
-      <c r="H11" s="105">
+      <c r="H11" s="114">
         <f t="shared" si="1"/>
         <v>202.86375999999996</v>
       </c>
-      <c r="I11" s="119">
+      <c r="I11" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6675,7 +6298,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K11" s="120">
+      <c r="K11" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6695,28 +6318,28 @@
       <c r="B12" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="94">
+      <c r="C12" s="87">
         <v>3.202</v>
       </c>
-      <c r="D12" s="83">
+      <c r="D12" s="80">
         <v>62.98</v>
       </c>
-      <c r="E12" s="93">
+      <c r="E12" s="112">
         <v>201.66195999999999</v>
       </c>
-      <c r="F12" s="106">
+      <c r="F12" s="118">
         <f>IFERROR(INDEX(usage!D:D, MATCH(CHECK!$B$3, usage!A:A, 0)) - INDEX(usage!D:D, MATCH(CHECK!$B$1, usage!A:A, 0)),"")</f>
         <v>3.202</v>
       </c>
-      <c r="G12" s="73">
+      <c r="G12" s="117">
         <f>INDEX(tariffs!4:4, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>62.98</v>
       </c>
-      <c r="H12" s="105">
+      <c r="H12" s="114">
         <f t="shared" si="1"/>
         <v>201.66195999999999</v>
       </c>
-      <c r="I12" s="119">
+      <c r="I12" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6724,7 +6347,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K12" s="120">
+      <c r="K12" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6744,28 +6367,28 @@
       <c r="B13" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="94">
+      <c r="C13" s="87">
         <v>3.202</v>
       </c>
-      <c r="D13" s="83">
+      <c r="D13" s="80">
         <v>44.12</v>
       </c>
-      <c r="E13" s="93">
+      <c r="E13" s="112">
         <v>141.27223999999998</v>
       </c>
-      <c r="F13" s="106">
+      <c r="F13" s="118">
         <f>F12</f>
         <v>3.202</v>
       </c>
-      <c r="G13" s="73">
+      <c r="G13" s="117">
         <f>INDEX(tariffs!5:5, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>44.12</v>
       </c>
-      <c r="H13" s="105">
+      <c r="H13" s="114">
         <f t="shared" si="1"/>
         <v>141.27223999999998</v>
       </c>
-      <c r="I13" s="119">
+      <c r="I13" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6773,7 +6396,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K13" s="120">
+      <c r="K13" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6794,28 +6417,28 @@
       <c r="B14" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="95">
+      <c r="C14" s="88">
         <v>6.952</v>
       </c>
-      <c r="D14" s="84">
+      <c r="D14" s="81">
         <v>227.18</v>
       </c>
-      <c r="E14" s="93">
+      <c r="E14" s="112">
         <v>1579.35536</v>
       </c>
-      <c r="F14" s="106">
+      <c r="F14" s="118">
         <f>IFERROR(C14,"")</f>
         <v>6.952</v>
       </c>
-      <c r="G14" s="73">
+      <c r="G14" s="117">
         <f>INDEX(tariffs!6:6, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>227.18</v>
       </c>
-      <c r="H14" s="105">
+      <c r="H14" s="114">
         <f t="shared" si="1"/>
         <v>1579.35536</v>
       </c>
-      <c r="I14" s="119">
+      <c r="I14" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6823,7 +6446,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K14" s="120">
+      <c r="K14" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6847,28 +6470,28 @@
       <c r="B15" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="94">
+      <c r="C15" s="87">
         <v>1.7152000000000001</v>
       </c>
-      <c r="D15" s="84">
+      <c r="D15" s="81">
         <v>3549.74</v>
       </c>
-      <c r="E15" s="93">
+      <c r="E15" s="112">
         <v>6535.25</v>
       </c>
-      <c r="F15" s="107">
+      <c r="F15" s="119">
         <f>IFERROR(C15,"")</f>
         <v>1.7152000000000001</v>
       </c>
-      <c r="G15" s="73">
+      <c r="G15" s="117">
         <f>INDEX(tariffs!7:7, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>3549.74</v>
       </c>
-      <c r="H15" s="105">
+      <c r="H15" s="114">
         <f t="shared" si="1"/>
         <v>6088.514048</v>
       </c>
-      <c r="I15" s="119">
+      <c r="I15" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6876,7 +6499,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K15" s="120">
+      <c r="K15" s="97">
         <f t="shared" si="0"/>
         <v>446.735952</v>
       </c>
@@ -6897,28 +6520,28 @@
       <c r="B16" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="94">
+      <c r="C16" s="87">
         <v>3</v>
       </c>
-      <c r="D16" s="83">
+      <c r="D16" s="80">
         <v>227.18</v>
       </c>
-      <c r="E16" s="93">
+      <c r="E16" s="112">
         <v>681.54</v>
       </c>
-      <c r="F16" s="106">
+      <c r="F16" s="118">
         <f t="shared" ref="F16:F20" si="4">IFERROR(C16,"")</f>
         <v>3</v>
       </c>
-      <c r="G16" s="73">
+      <c r="G16" s="117">
         <f>INDEX(tariffs!6:6, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>227.18</v>
       </c>
-      <c r="H16" s="105">
+      <c r="H16" s="114">
         <f t="shared" si="1"/>
         <v>681.54</v>
       </c>
-      <c r="I16" s="119">
+      <c r="I16" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6926,7 +6549,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K16" s="120">
+      <c r="K16" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6947,28 +6570,28 @@
       <c r="B17" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="94">
+      <c r="C17" s="87">
         <v>0.68</v>
       </c>
-      <c r="D17" s="83">
+      <c r="D17" s="80">
         <v>62.98</v>
       </c>
-      <c r="E17" s="93">
+      <c r="E17" s="112">
         <v>42.8264</v>
       </c>
-      <c r="F17" s="106">
+      <c r="F17" s="118">
         <f t="shared" si="4"/>
         <v>0.68</v>
       </c>
-      <c r="G17" s="73">
+      <c r="G17" s="117">
         <f>INDEX(tariffs!4:4, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>62.98</v>
       </c>
-      <c r="H17" s="105">
+      <c r="H17" s="114">
         <f t="shared" si="1"/>
         <v>42.8264</v>
       </c>
-      <c r="I17" s="119">
+      <c r="I17" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -6976,7 +6599,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K17" s="120">
+      <c r="K17" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7000,28 +6623,28 @@
       <c r="B18" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="94">
+      <c r="C18" s="87">
         <v>1.36</v>
       </c>
-      <c r="D18" s="84">
+      <c r="D18" s="81">
         <v>62.98</v>
       </c>
-      <c r="E18" s="93">
+      <c r="E18" s="112">
         <v>85.652799999999999</v>
       </c>
-      <c r="F18" s="106">
+      <c r="F18" s="118">
         <f t="shared" si="4"/>
         <v>1.36</v>
       </c>
-      <c r="G18" s="73">
+      <c r="G18" s="117">
         <f>INDEX(tariffs!4:4, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>62.98</v>
       </c>
-      <c r="H18" s="105">
+      <c r="H18" s="114">
         <f t="shared" si="1"/>
         <v>85.652799999999999</v>
       </c>
-      <c r="I18" s="119">
+      <c r="I18" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -7029,7 +6652,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K18" s="120">
+      <c r="K18" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7053,28 +6676,28 @@
       <c r="B19" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="94">
+      <c r="C19" s="87">
         <v>1.36</v>
       </c>
-      <c r="D19" s="84">
+      <c r="D19" s="81">
         <v>44.12</v>
       </c>
-      <c r="E19" s="93">
+      <c r="E19" s="112">
         <v>60.0032</v>
       </c>
-      <c r="F19" s="106">
+      <c r="F19" s="118">
         <f t="shared" si="4"/>
         <v>1.36</v>
       </c>
-      <c r="G19" s="73">
+      <c r="G19" s="117">
         <f>INDEX(tariffs!5:5, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>44.12</v>
       </c>
-      <c r="H19" s="105">
+      <c r="H19" s="114">
         <f t="shared" si="1"/>
         <v>60.0032</v>
       </c>
-      <c r="I19" s="119">
+      <c r="I19" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -7082,7 +6705,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K19" s="120">
+      <c r="K19" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7106,28 +6729,28 @@
       <c r="B20" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="94">
+      <c r="C20" s="87">
         <v>26.83</v>
       </c>
-      <c r="D20" s="83">
+      <c r="D20" s="80">
         <v>4.2</v>
       </c>
-      <c r="E20" s="93">
+      <c r="E20" s="112">
         <v>112.68599999999999</v>
       </c>
-      <c r="F20" s="108">
+      <c r="F20" s="120">
         <f t="shared" si="4"/>
         <v>26.83</v>
       </c>
-      <c r="G20" s="73">
+      <c r="G20" s="117">
         <f>INDEX(tariffs!2:2, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>4.2</v>
       </c>
-      <c r="H20" s="105">
+      <c r="H20" s="114">
         <f t="shared" si="1"/>
         <v>112.68599999999999</v>
       </c>
-      <c r="I20" s="119">
+      <c r="I20" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -7135,7 +6758,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K20" s="120">
+      <c r="K20" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7159,28 +6782,28 @@
       <c r="B21" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="94">
+      <c r="C21" s="87">
         <v>55.2</v>
       </c>
-      <c r="D21" s="83">
+      <c r="D21" s="80">
         <v>11.08</v>
       </c>
-      <c r="E21" s="93">
+      <c r="E21" s="112">
         <v>611.61599999999999</v>
       </c>
-      <c r="F21" s="109">
+      <c r="F21" s="121">
         <f>IFERROR(info!$B$7,"")</f>
         <v>55.2</v>
       </c>
-      <c r="G21" s="73">
+      <c r="G21" s="117">
         <f>INDEX(tariffs!8:8, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>11.08</v>
       </c>
-      <c r="H21" s="105">
+      <c r="H21" s="114">
         <f t="shared" si="1"/>
         <v>611.61599999999999</v>
       </c>
-      <c r="I21" s="119">
+      <c r="I21" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -7188,7 +6811,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K21" s="120">
+      <c r="K21" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7209,28 +6832,28 @@
       <c r="B22" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="94">
+      <c r="C22" s="87">
         <v>55.2</v>
       </c>
-      <c r="D22" s="83">
+      <c r="D22" s="80">
         <v>5.98</v>
       </c>
-      <c r="E22" s="93">
+      <c r="E22" s="112">
         <v>330.09600000000006</v>
       </c>
-      <c r="F22" s="109">
+      <c r="F22" s="121">
         <f>IFERROR(info!$B$7,"")</f>
         <v>55.2</v>
       </c>
-      <c r="G22" s="73">
+      <c r="G22" s="117">
         <f>INDEX(tariffs!9:9, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>5.98</v>
       </c>
-      <c r="H22" s="105">
+      <c r="H22" s="114">
         <f t="shared" si="1"/>
         <v>330.09600000000006</v>
       </c>
-      <c r="I22" s="119">
+      <c r="I22" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -7238,7 +6861,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K22" s="120">
+      <c r="K22" s="97">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7259,28 +6882,28 @@
       <c r="B23" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="94">
+      <c r="C23" s="87">
         <v>2</v>
       </c>
-      <c r="D23" s="83">
+      <c r="D23" s="80">
         <v>158</v>
       </c>
-      <c r="E23" s="93">
+      <c r="E23" s="112">
         <v>316</v>
       </c>
-      <c r="F23" s="104">
+      <c r="F23" s="116">
         <f>IFERROR(info!$B$6,"")</f>
         <v>2</v>
       </c>
-      <c r="G23" s="73">
+      <c r="G23" s="117">
         <f>INDEX(tariffs!10:10, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>161.52257251624999</v>
       </c>
-      <c r="H23" s="105">
+      <c r="H23" s="114">
         <f t="shared" si="1"/>
         <v>323.04514503249999</v>
       </c>
-      <c r="I23" s="119">
+      <c r="I23" s="96">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -7288,7 +6911,7 @@
         <f t="shared" si="0"/>
         <v>-3.5225725162499941</v>
       </c>
-      <c r="K23" s="120">
+      <c r="K23" s="97">
         <f t="shared" si="0"/>
         <v>-7.0451450324999882</v>
       </c>
@@ -7312,36 +6935,36 @@
       <c r="B24" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="96">
+      <c r="C24" s="89">
         <v>55.2</v>
       </c>
-      <c r="D24" s="97">
+      <c r="D24" s="90">
         <v>15.15</v>
       </c>
-      <c r="E24" s="98">
+      <c r="E24" s="113">
         <v>836.28000000000009</v>
       </c>
-      <c r="F24" s="110">
+      <c r="F24" s="122">
         <f>IFERROR(info!$B$7,"")</f>
         <v>55.2</v>
       </c>
-      <c r="G24" s="111">
+      <c r="G24" s="123">
         <f>INDEX(tariffs!11:11, MATCH(CHECK!$B$3,tariffs!$1:$1, 0))</f>
         <v>15.15</v>
       </c>
-      <c r="H24" s="112">
+      <c r="H24" s="115">
         <f t="shared" si="1"/>
         <v>836.28000000000009</v>
       </c>
-      <c r="I24" s="121">
+      <c r="I24" s="98">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J24" s="122">
+      <c r="J24" s="99">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K24" s="123">
+      <c r="K24" s="100">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -7393,7 +7016,7 @@
         <v>452.29080696750003</v>
       </c>
       <c r="L26" s="3" t="str">
-        <f t="shared" ref="L10:L32" si="5">IF(ABS(K26)&lt;=1,"✔ ОК",IF(K26&gt;1,"❗ Превышение","❗ Недосчет"))</f>
+        <f t="shared" ref="L26" si="5">IF(ABS(K26)&lt;=1,"✔ ОК",IF(K26&gt;1,"❗ Превышение","❗ Недосчет"))</f>
         <v>❗ Превышение</v>
       </c>
       <c r="M26" s="40"/>
@@ -7543,33 +7166,33 @@
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="I7:K7"/>
   </mergeCells>
+  <conditionalFormatting sqref="I9:K24 K26 K28:K32">
+    <cfRule type="expression" dxfId="4" priority="1">
+      <formula>AND($K9&lt;&gt;"",$K9&lt;-0.1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>AND($K9&lt;&gt;"",$K9&gt;0.1)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L1:L24 L26:L1048576">
-    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="✔ ОК">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="❗ Недосчет">
+      <formula>NOT(ISERROR(SEARCH("❗ Недосчет",L1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="❗ Превышение">
+      <formula>NOT(ISERROR(SEARCH("❗ Превышение",L1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="✔ ОК">
       <formula>NOT(ISERROR(SEARCH("✔ ОК",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="❗ Превышение">
-      <formula>NOT(ISERROR(SEARCH("❗ Превышение",L1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="❗ Недосчет">
-      <formula>NOT(ISERROR(SEARCH("❗ Недосчет",L1)))</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I9:K24 K26 K28:K32">
-    <cfRule type="expression" dxfId="6" priority="2">
-      <formula>AND($K9&lt;&gt;"",$K9&gt;0.1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="1">
-      <formula>AND($K9&lt;&gt;"",$K9&lt;-0.1)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:D9" xr:uid="{EEAF0B01-A716-45A5-80B9-6D59D6176D06}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="4">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6E04C081-2925-4DDE-9260-64EC5751E787}">
           <x14:formula1>
             <xm:f>helper!$E$2:$E$10</xm:f>
@@ -7657,11 +7280,11 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
     </row>
     <row r="2" spans="1:28" s="11" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="50" t="s">
@@ -7913,13 +7536,13 @@
       <c r="K25"/>
     </row>
     <row r="26" spans="2:11" ht="16" x14ac:dyDescent="0.4">
-      <c r="B26" s="79" t="s">
+      <c r="B26" s="111" t="s">
         <v>120</v>
       </c>
-      <c r="C26" s="79"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="79"/>
-      <c r="F26" s="79"/>
+      <c r="C26" s="111"/>
+      <c r="D26" s="111"/>
+      <c r="E26" s="111"/>
+      <c r="F26" s="111"/>
       <c r="G26"/>
       <c r="H26"/>
       <c r="I26"/>
@@ -8978,216 +8601,216 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="76">
+      <c r="A2" s="75">
         <v>45627</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="76">
+      <c r="A3" s="75">
         <v>45658</v>
       </c>
-      <c r="B3" s="81"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
     </row>
     <row r="4" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="76">
+      <c r="A4" s="75">
         <v>45689</v>
       </c>
-      <c r="B4" s="81"/>
-      <c r="C4" s="80"/>
-      <c r="D4" s="80"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="77"/>
     </row>
     <row r="5" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="76">
+      <c r="A5" s="75">
         <v>45717</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
     </row>
     <row r="6" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="76">
+      <c r="A6" s="75">
         <v>45748</v>
       </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="80"/>
-      <c r="D6" s="80"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="77"/>
     </row>
     <row r="7" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="76">
+      <c r="A7" s="75">
         <v>45778</v>
       </c>
-      <c r="B7" s="81"/>
-      <c r="C7" s="80"/>
-      <c r="D7" s="80"/>
+      <c r="B7" s="78"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="77"/>
     </row>
     <row r="8" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="76">
+      <c r="A8" s="75">
         <v>45809</v>
       </c>
-      <c r="B8" s="81"/>
-      <c r="C8" s="80"/>
-      <c r="D8" s="80"/>
+      <c r="B8" s="78"/>
+      <c r="C8" s="77"/>
+      <c r="D8" s="77"/>
     </row>
     <row r="9" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="76">
+      <c r="A9" s="75">
         <v>45839</v>
       </c>
-      <c r="B9" s="81"/>
-      <c r="C9" s="80"/>
-      <c r="D9" s="80"/>
+      <c r="B9" s="78"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
     </row>
     <row r="10" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="76">
+      <c r="A10" s="75">
         <v>45870</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="80"/>
-      <c r="D10" s="80"/>
+      <c r="B10" s="78"/>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
     </row>
     <row r="11" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="76">
+      <c r="A11" s="75">
         <v>45901</v>
       </c>
-      <c r="B11" s="81"/>
-      <c r="C11" s="80"/>
-      <c r="D11" s="80"/>
+      <c r="B11" s="78"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
     </row>
     <row r="12" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="76">
+      <c r="A12" s="75">
         <v>45931</v>
       </c>
-      <c r="B12" s="81"/>
-      <c r="C12" s="80"/>
-      <c r="D12" s="80"/>
+      <c r="B12" s="78"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
     </row>
     <row r="13" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="76">
+      <c r="A13" s="75">
         <v>45962</v>
       </c>
-      <c r="B13" s="81"/>
-      <c r="C13" s="80"/>
-      <c r="D13" s="80"/>
+      <c r="B13" s="78"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
     </row>
     <row r="14" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="76">
+      <c r="A14" s="75">
         <v>45992</v>
       </c>
-      <c r="B14" s="81"/>
-      <c r="C14" s="80"/>
-      <c r="D14" s="80"/>
+      <c r="B14" s="78"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
     </row>
     <row r="15" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="76">
+      <c r="A15" s="75">
         <v>46023</v>
       </c>
-      <c r="B15" s="81">
+      <c r="B15" s="78">
         <v>1562</v>
       </c>
-      <c r="C15" s="80">
+      <c r="C15" s="77">
         <v>8.3000000000000007</v>
       </c>
-      <c r="D15" s="80">
+      <c r="D15" s="77">
         <v>9.1229999999999993</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="76">
+      <c r="A16" s="75">
         <v>46054</v>
       </c>
-      <c r="B16" s="81">
+      <c r="B16" s="78">
         <v>1763</v>
       </c>
-      <c r="C16" s="80">
+      <c r="C16" s="77">
         <v>12.898</v>
       </c>
-      <c r="D16" s="80">
+      <c r="D16" s="77">
         <v>12.324999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="76">
+      <c r="A17" s="75">
         <v>46082</v>
       </c>
-      <c r="B17" s="81"/>
-      <c r="C17" s="80"/>
-      <c r="D17" s="80"/>
+      <c r="B17" s="78"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="77"/>
     </row>
     <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="76">
+      <c r="A18" s="75">
         <v>46113</v>
       </c>
-      <c r="B18" s="81"/>
-      <c r="C18" s="80"/>
-      <c r="D18" s="80"/>
+      <c r="B18" s="78"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
     </row>
     <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="76">
+      <c r="A19" s="75">
         <v>46143</v>
       </c>
-      <c r="B19" s="81"/>
-      <c r="C19" s="80"/>
-      <c r="D19" s="80"/>
+      <c r="B19" s="78"/>
+      <c r="C19" s="77"/>
+      <c r="D19" s="77"/>
     </row>
     <row r="20" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="76">
+      <c r="A20" s="75">
         <v>46174</v>
       </c>
-      <c r="B20" s="81"/>
-      <c r="C20" s="80"/>
-      <c r="D20" s="80"/>
+      <c r="B20" s="78"/>
+      <c r="C20" s="77"/>
+      <c r="D20" s="77"/>
     </row>
     <row r="21" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="76">
+      <c r="A21" s="75">
         <v>46204</v>
       </c>
-      <c r="B21" s="81"/>
-      <c r="C21" s="80"/>
-      <c r="D21" s="80"/>
+      <c r="B21" s="78"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
     </row>
     <row r="22" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="76">
+      <c r="A22" s="75">
         <v>46235</v>
       </c>
-      <c r="B22" s="81"/>
-      <c r="C22" s="80"/>
-      <c r="D22" s="80"/>
+      <c r="B22" s="78"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
     </row>
     <row r="23" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="76">
+      <c r="A23" s="75">
         <v>46266</v>
       </c>
-      <c r="B23" s="81"/>
-      <c r="C23" s="80"/>
-      <c r="D23" s="80"/>
+      <c r="B23" s="78"/>
+      <c r="C23" s="77"/>
+      <c r="D23" s="77"/>
     </row>
     <row r="24" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="76">
+      <c r="A24" s="75">
         <v>46296</v>
       </c>
-      <c r="B24" s="81"/>
-      <c r="C24" s="80"/>
-      <c r="D24" s="80"/>
+      <c r="B24" s="78"/>
+      <c r="C24" s="77"/>
+      <c r="D24" s="77"/>
     </row>
     <row r="25" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="76">
+      <c r="A25" s="75">
         <v>46327</v>
       </c>
-      <c r="B25" s="81"/>
-      <c r="C25" s="80"/>
-      <c r="D25" s="80"/>
+      <c r="B25" s="78"/>
+      <c r="C25" s="77"/>
+      <c r="D25" s="77"/>
     </row>
     <row r="26" spans="1:4" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="76">
+      <c r="A26" s="75">
         <v>46357</v>
       </c>
-      <c r="B26" s="81"/>
-      <c r="C26" s="80"/>
-      <c r="D26" s="80"/>
+      <c r="B26" s="78"/>
+      <c r="C26" s="77"/>
+      <c r="D26" s="77"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9232,112 +8855,112 @@
       <c r="B1" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="82">
+      <c r="C1" s="79">
         <v>45292</v>
       </c>
-      <c r="D1" s="82">
+      <c r="D1" s="79">
         <v>45323</v>
       </c>
-      <c r="E1" s="82">
+      <c r="E1" s="79">
         <v>45352</v>
       </c>
-      <c r="F1" s="82">
+      <c r="F1" s="79">
         <v>45383</v>
       </c>
-      <c r="G1" s="82">
+      <c r="G1" s="79">
         <v>45413</v>
       </c>
-      <c r="H1" s="82">
+      <c r="H1" s="79">
         <v>45444</v>
       </c>
-      <c r="I1" s="82">
+      <c r="I1" s="79">
         <v>45474</v>
       </c>
-      <c r="J1" s="82">
+      <c r="J1" s="79">
         <v>45505</v>
       </c>
-      <c r="K1" s="82">
+      <c r="K1" s="79">
         <v>45536</v>
       </c>
-      <c r="L1" s="82">
+      <c r="L1" s="79">
         <v>45566</v>
       </c>
-      <c r="M1" s="82">
+      <c r="M1" s="79">
         <v>45597</v>
       </c>
-      <c r="N1" s="82">
+      <c r="N1" s="79">
         <v>45627</v>
       </c>
-      <c r="O1" s="82">
+      <c r="O1" s="79">
         <v>45658</v>
       </c>
-      <c r="P1" s="82">
+      <c r="P1" s="79">
         <v>45689</v>
       </c>
-      <c r="Q1" s="82">
+      <c r="Q1" s="79">
         <v>45717</v>
       </c>
-      <c r="R1" s="82">
+      <c r="R1" s="79">
         <v>45748</v>
       </c>
-      <c r="S1" s="82">
+      <c r="S1" s="79">
         <v>45778</v>
       </c>
-      <c r="T1" s="82">
+      <c r="T1" s="79">
         <v>45809</v>
       </c>
-      <c r="U1" s="82">
+      <c r="U1" s="79">
         <v>45839</v>
       </c>
-      <c r="V1" s="82">
+      <c r="V1" s="79">
         <v>45870</v>
       </c>
-      <c r="W1" s="82">
+      <c r="W1" s="79">
         <v>45901</v>
       </c>
-      <c r="X1" s="82">
+      <c r="X1" s="79">
         <v>45931</v>
       </c>
-      <c r="Y1" s="82">
+      <c r="Y1" s="79">
         <v>45962</v>
       </c>
-      <c r="Z1" s="82">
+      <c r="Z1" s="79">
         <v>45992</v>
       </c>
-      <c r="AA1" s="82">
+      <c r="AA1" s="79">
         <v>46023</v>
       </c>
-      <c r="AB1" s="82">
+      <c r="AB1" s="79">
         <v>46054</v>
       </c>
-      <c r="AC1" s="82">
+      <c r="AC1" s="79">
         <v>46082</v>
       </c>
-      <c r="AD1" s="82">
+      <c r="AD1" s="79">
         <v>46113</v>
       </c>
-      <c r="AE1" s="82">
+      <c r="AE1" s="79">
         <v>46143</v>
       </c>
-      <c r="AF1" s="82">
+      <c r="AF1" s="79">
         <v>46174</v>
       </c>
-      <c r="AG1" s="82">
+      <c r="AG1" s="79">
         <v>46204</v>
       </c>
-      <c r="AH1" s="82">
+      <c r="AH1" s="79">
         <v>46235</v>
       </c>
-      <c r="AI1" s="82">
+      <c r="AI1" s="79">
         <v>46266</v>
       </c>
-      <c r="AJ1" s="82">
+      <c r="AJ1" s="79">
         <v>46296</v>
       </c>
-      <c r="AK1" s="82">
+      <c r="AK1" s="79">
         <v>46327</v>
       </c>
-      <c r="AL1" s="82">
+      <c r="AL1" s="79">
         <v>46357</v>
       </c>
       <c r="AM1" s="51" t="s">
@@ -9462,7 +9085,7 @@
       <c r="AM2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="AN2" s="85" t="s">
+      <c r="AN2" s="82" t="s">
         <v>148</v>
       </c>
     </row>
@@ -9701,7 +9324,7 @@
       <c r="AM4" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="AN4" s="85" t="s">
+      <c r="AN4" s="82" t="s">
         <v>149</v>
       </c>
     </row>
@@ -10444,7 +10067,7 @@
       <c r="AM10" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="AN10" s="85" t="s">
+      <c r="AN10" s="82" t="s">
         <v>150</v>
       </c>
     </row>
@@ -10566,7 +10189,7 @@
       <c r="AM11" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="AN11" s="85" t="s">
+      <c r="AN11" s="82" t="s">
         <v>151</v>
       </c>
     </row>
@@ -11731,27 +11354,27 @@
       <c r="B38" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C38" s="86">
+      <c r="C38" s="83">
         <f>C37*C36*C35/12</f>
         <v>132.34105224799995</v>
       </c>
-      <c r="I38" s="86">
+      <c r="I38" s="83">
         <f>I37*I36*I35/12</f>
         <v>144.91470621139999</v>
       </c>
-      <c r="O38" s="86">
+      <c r="O38" s="83">
         <f>O37*O36*O35/12</f>
         <v>171.78310199199996</v>
       </c>
-      <c r="U38" s="86">
+      <c r="U38" s="83">
         <f>U37*U36*U35/12</f>
         <v>158.82299893999999</v>
       </c>
-      <c r="AA38" s="86">
-        <f t="shared" ref="AA38:AB38" si="6">AA37*AA36*AA35/12</f>
+      <c r="AA38" s="83">
+        <f t="shared" ref="AA38" si="6">AA37*AA36*AA35/12</f>
         <v>161.52257251624999</v>
       </c>
-      <c r="AG38" s="86">
+      <c r="AG38" s="83">
         <f>AG37*AG36*AG35/12</f>
         <v>161.52257251624999</v>
       </c>

</xml_diff>